<commit_message>
[auto-snapshot] 2026-04-29 20:00 | onda-hompage | 60 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_nail/용인_네일샵.xlsx
+++ b/naver-place-crawler/results_nail/용인_네일샵.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V727"/>
+  <dimension ref="A1:V753"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -67221,34 +67221,30 @@
     <row r="725">
       <c r="A725" t="inlineStr">
         <is>
-          <t>미용실</t>
+          <t>네일아트,네일샵</t>
         </is>
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>함스헤어</t>
-        </is>
-      </c>
-      <c r="C725" t="inlineStr">
-        <is>
-          <t>rose74741@naver.com</t>
-        </is>
-      </c>
+          <t>손네일</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr"/>
       <c r="D725" t="inlineStr"/>
       <c r="E725" t="inlineStr">
         <is>
-          <t>0507-1374-7910</t>
+          <t>0507-1325-4489</t>
         </is>
       </c>
       <c r="F725" t="inlineStr"/>
       <c r="G725" t="inlineStr">
         <is>
-          <t>경기도 용인시 처인구 유림로 148-4</t>
+          <t>경기도 용인시 기흥구 죽전로15번길 3-20</t>
         </is>
       </c>
       <c r="H725" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>http://www.instagram.com/kim_sonnail</t>
         </is>
       </c>
       <c r="I725" t="inlineStr">
@@ -67258,7 +67254,7 @@
       </c>
       <c r="J725" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K725" t="inlineStr">
@@ -67279,17 +67275,17 @@
       </c>
       <c r="O725" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P725" t="n">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="Q725" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R725" t="n">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="S725" t="inlineStr">
         <is>
@@ -67298,12 +67294,12 @@
       </c>
       <c r="T725" t="inlineStr">
         <is>
-          <t>37036591</t>
+          <t>35316312</t>
         </is>
       </c>
       <c r="U725" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/37036591</t>
+          <t>https://m.place.naver.com/place/35316312</t>
         </is>
       </c>
       <c r="V725" t="inlineStr">
@@ -67315,34 +67311,34 @@
     <row r="726">
       <c r="A726" t="inlineStr">
         <is>
-          <t>인테리어디자인</t>
+          <t>네일아트,네일샵</t>
         </is>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>스페이스와이 SPACE Y</t>
+          <t>네일드로우</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
         <is>
-          <t>yonseiblog@naver.com</t>
+          <t>ssuna0116@naver.com</t>
         </is>
       </c>
       <c r="D726" t="inlineStr"/>
       <c r="E726" t="inlineStr">
         <is>
-          <t>0507-1396-3851</t>
+          <t>0507-1483-2243</t>
         </is>
       </c>
       <c r="F726" t="inlineStr"/>
       <c r="G726" t="inlineStr">
         <is>
-          <t>경기도 화성시 동탄구 동탄대로 599 303호</t>
+          <t>경기도 용인시 기흥구 중부대로 184 힉스유타워 상가동 1층 169-2호</t>
         </is>
       </c>
       <c r="H726" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>http://instagram.com/nail_draw_jin</t>
         </is>
       </c>
       <c r="I726" t="inlineStr">
@@ -67352,7 +67348,7 @@
       </c>
       <c r="J726" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K726" t="inlineStr">
@@ -67368,22 +67364,22 @@
       <c r="M726" t="inlineStr"/>
       <c r="N726" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O726" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P726" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q726" t="n">
         <v>0</v>
       </c>
       <c r="R726" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S726" t="inlineStr">
         <is>
@@ -67392,12 +67388,12 @@
       </c>
       <c r="T726" t="inlineStr">
         <is>
-          <t>1315149633</t>
+          <t>1439291395</t>
         </is>
       </c>
       <c r="U726" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1315149633</t>
+          <t>https://m.place.naver.com/place/1439291395</t>
         </is>
       </c>
       <c r="V726" t="inlineStr">
@@ -67409,26 +67405,30 @@
     <row r="727">
       <c r="A727" t="inlineStr">
         <is>
-          <t>인테리어디자인</t>
+          <t>네일아트,네일샵</t>
         </is>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>웰디자인</t>
+          <t>네일리르</t>
         </is>
       </c>
       <c r="C727" t="inlineStr"/>
       <c r="D727" t="inlineStr"/>
-      <c r="E727" t="inlineStr"/>
+      <c r="E727" t="inlineStr">
+        <is>
+          <t>0507-1469-2295</t>
+        </is>
+      </c>
       <c r="F727" t="inlineStr"/>
       <c r="G727" t="inlineStr">
         <is>
-          <t>경기도 용인시 수지구 풍덕천로 52</t>
+          <t>경기도 용인시 기흥구 죽전로 23 2층 202호</t>
         </is>
       </c>
       <c r="H727" t="inlineStr">
         <is>
-          <t>http://www.instagram.com/well_design24</t>
+          <t>https://www.instagram.com/nail_rire_</t>
         </is>
       </c>
       <c r="I727" t="inlineStr">
@@ -67463,30 +67463,2438 @@
         </is>
       </c>
       <c r="P727" t="n">
+        <v>376</v>
+      </c>
+      <c r="Q727" t="n">
+        <v>19</v>
+      </c>
+      <c r="R727" t="n">
+        <v>395</v>
+      </c>
+      <c r="S727" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T727" t="inlineStr">
+        <is>
+          <t>1370128010</t>
+        </is>
+      </c>
+      <c r="U727" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1370128010</t>
+        </is>
+      </c>
+      <c r="V727" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>에이치네일</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>remon103@naver.com</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr"/>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>0507-1318-3991</t>
+        </is>
+      </c>
+      <c r="F728" t="inlineStr"/>
+      <c r="G728" t="inlineStr">
+        <is>
+          <t>경기도 화성시 동탄구 동탄대로5길 15 5층 5026호</t>
+        </is>
+      </c>
+      <c r="H728" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J728" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K728" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L728" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M728" t="inlineStr"/>
+      <c r="N728" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O728" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P728" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q728" t="n">
         <v>1</v>
       </c>
-      <c r="Q727" t="n">
+      <c r="R728" t="n">
+        <v>14</v>
+      </c>
+      <c r="S728" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T728" t="inlineStr">
+        <is>
+          <t>2017869489</t>
+        </is>
+      </c>
+      <c r="U728" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/2017869489</t>
+        </is>
+      </c>
+      <c r="V728" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>뮤제네일 수원영통점</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>sarsh1205@naver.com</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr"/>
+      <c r="E729" t="inlineStr">
+        <is>
+          <t>0507-1389-8681</t>
+        </is>
+      </c>
+      <c r="F729" t="inlineStr"/>
+      <c r="G729" t="inlineStr">
+        <is>
+          <t>경기도 수원시 영통구 덕영대로 1699 303A호</t>
+        </is>
+      </c>
+      <c r="H729" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/musee_nail?igsh=MTk1aDdqYTdiaGt5cA%3D%3D&amp;utm_source=qr</t>
+        </is>
+      </c>
+      <c r="I729" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J729" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K729" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L729" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M729" t="inlineStr"/>
+      <c r="N729" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O729" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P729" t="n">
+        <v>286</v>
+      </c>
+      <c r="Q729" t="n">
+        <v>50</v>
+      </c>
+      <c r="R729" t="n">
+        <v>336</v>
+      </c>
+      <c r="S729" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T729" t="inlineStr">
+        <is>
+          <t>2045620652</t>
+        </is>
+      </c>
+      <c r="U729" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/2045620652</t>
+        </is>
+      </c>
+      <c r="V729" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>네일가든</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>minee_94@naver.com</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr"/>
+      <c r="E730" t="inlineStr">
+        <is>
+          <t>031-896-4141</t>
+        </is>
+      </c>
+      <c r="F730" t="inlineStr"/>
+      <c r="G730" t="inlineStr">
+        <is>
+          <t>경기도 용인시 수지구 현암로 153 건영타운 1층</t>
+        </is>
+      </c>
+      <c r="H730" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J730" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K730" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L730" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M730" t="inlineStr"/>
+      <c r="N730" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O730" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P730" t="n">
         <v>0</v>
       </c>
-      <c r="R727" t="n">
+      <c r="Q730" t="n">
+        <v>0</v>
+      </c>
+      <c r="R730" t="n">
+        <v>0</v>
+      </c>
+      <c r="S730" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T730" t="inlineStr">
+        <is>
+          <t>34762150</t>
+        </is>
+      </c>
+      <c r="U730" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/34762150</t>
+        </is>
+      </c>
+      <c r="V730" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>네일쥬르</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>laumi22@naver.com</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr"/>
+      <c r="E731" t="inlineStr">
+        <is>
+          <t>0507-1468-2788</t>
+        </is>
+      </c>
+      <c r="F731" t="inlineStr"/>
+      <c r="G731" t="inlineStr">
+        <is>
+          <t>경기도 용인시 수지구 현암로 148 스카이프라자 3층 302호</t>
+        </is>
+      </c>
+      <c r="H731" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nailjours/</t>
+        </is>
+      </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J731" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K731" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L731" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M731" t="inlineStr"/>
+      <c r="N731" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O731" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P731" t="n">
+        <v>246</v>
+      </c>
+      <c r="Q731" t="n">
+        <v>8</v>
+      </c>
+      <c r="R731" t="n">
+        <v>254</v>
+      </c>
+      <c r="S731" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T731" t="inlineStr">
+        <is>
+          <t>1186917891</t>
+        </is>
+      </c>
+      <c r="U731" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1186917891</t>
+        </is>
+      </c>
+      <c r="V731" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>에이네일</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr"/>
+      <c r="D732" t="inlineStr"/>
+      <c r="E732" t="inlineStr"/>
+      <c r="F732" t="inlineStr"/>
+      <c r="G732" t="inlineStr">
+        <is>
+          <t>경기도 용인시 처인구 남사읍 한숲로 45 B동 4층 417호</t>
+        </is>
+      </c>
+      <c r="H732" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/a.nail_hansoop</t>
+        </is>
+      </c>
+      <c r="I732" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J732" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K732" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L732" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M732" t="inlineStr"/>
+      <c r="N732" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O732" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P732" t="n">
+        <v>47</v>
+      </c>
+      <c r="Q732" t="n">
+        <v>0</v>
+      </c>
+      <c r="R732" t="n">
+        <v>47</v>
+      </c>
+      <c r="S732" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T732" t="inlineStr">
+        <is>
+          <t>1604007860</t>
+        </is>
+      </c>
+      <c r="U732" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1604007860</t>
+        </is>
+      </c>
+      <c r="V732" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>더와이네일</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>msbhaha@naver.com</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr"/>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>0507-1418-0427</t>
+        </is>
+      </c>
+      <c r="F733" t="inlineStr"/>
+      <c r="G733" t="inlineStr">
+        <is>
+          <t>경기도 용인시 처인구 명지로 24 the럭스나인 204로 더와이네일</t>
+        </is>
+      </c>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>http://instagram.com/the_y_nail_</t>
+        </is>
+      </c>
+      <c r="I733" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J733" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K733" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L733" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M733" t="inlineStr"/>
+      <c r="N733" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O733" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P733" t="n">
+        <v>424</v>
+      </c>
+      <c r="Q733" t="n">
+        <v>7</v>
+      </c>
+      <c r="R733" t="n">
+        <v>431</v>
+      </c>
+      <c r="S733" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T733" t="inlineStr">
+        <is>
+          <t>1853278359</t>
+        </is>
+      </c>
+      <c r="U733" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1853278359</t>
+        </is>
+      </c>
+      <c r="V733" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>샤네일</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>jgy5220@naver.com</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr"/>
+      <c r="E734" t="inlineStr">
+        <is>
+          <t>0507-1314-1643</t>
+        </is>
+      </c>
+      <c r="F734" t="inlineStr"/>
+      <c r="G734" t="inlineStr">
+        <is>
+          <t>경기도 용인시 처인구 금학로 442</t>
+        </is>
+      </c>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>http://instagram.com/cha.nail__</t>
+        </is>
+      </c>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J734" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K734" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L734" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M734" t="inlineStr"/>
+      <c r="N734" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O734" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P734" t="n">
+        <v>37</v>
+      </c>
+      <c r="Q734" t="n">
+        <v>10</v>
+      </c>
+      <c r="R734" t="n">
+        <v>47</v>
+      </c>
+      <c r="S734" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T734" t="inlineStr">
+        <is>
+          <t>1311854053</t>
+        </is>
+      </c>
+      <c r="U734" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1311854053</t>
+        </is>
+      </c>
+      <c r="V734" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>네일도</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>sungunara226@naver.com</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr"/>
+      <c r="E735" t="inlineStr">
+        <is>
+          <t>0507-1359-5645</t>
+        </is>
+      </c>
+      <c r="F735" t="inlineStr"/>
+      <c r="G735" t="inlineStr">
+        <is>
+          <t>경기도 용인시 수지구 광교마을로 54 광교 SB타운 307호</t>
+        </is>
+      </c>
+      <c r="H735" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/__nail.do__?igsh=MWZmMm9kYzY0bDYxdA%3D%3D&amp;utm_source=qr</t>
+        </is>
+      </c>
+      <c r="I735" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J735" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K735" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L735" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M735" t="inlineStr"/>
+      <c r="N735" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O735" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P735" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q735" t="n">
+        <v>6</v>
+      </c>
+      <c r="R735" t="n">
+        <v>46</v>
+      </c>
+      <c r="S735" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T735" t="inlineStr">
+        <is>
+          <t>2034335729</t>
+        </is>
+      </c>
+      <c r="U735" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/2034335729</t>
+        </is>
+      </c>
+      <c r="V735" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>레푸스 수지구청점</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>aden727@naver.com</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr"/>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>0507-1439-3384</t>
+        </is>
+      </c>
+      <c r="F736" t="inlineStr"/>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>경기도 용인시 수지구 풍덕천로 122 4층 405-2호</t>
+        </is>
+      </c>
+      <c r="H736" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/aden727</t>
+        </is>
+      </c>
+      <c r="I736" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J736" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K736" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L736" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M736" t="inlineStr"/>
+      <c r="N736" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O736" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P736" t="n">
+        <v>1117</v>
+      </c>
+      <c r="Q736" t="n">
+        <v>903</v>
+      </c>
+      <c r="R736" t="n">
+        <v>2020</v>
+      </c>
+      <c r="S736" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T736" t="inlineStr">
+        <is>
+          <t>1846095043</t>
+        </is>
+      </c>
+      <c r="U736" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1846095043</t>
+        </is>
+      </c>
+      <c r="V736" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>네일엘로이 동탄</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>gu17190@naver.com</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr"/>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>0507-1310-1386</t>
+        </is>
+      </c>
+      <c r="F737" t="inlineStr"/>
+      <c r="G737" t="inlineStr">
+        <is>
+          <t>경기도 화성시 동탄구 동탄공원로3길 32-6 1층 103호</t>
+        </is>
+      </c>
+      <c r="H737" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nail_elroy</t>
+        </is>
+      </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J737" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K737" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L737" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M737" t="inlineStr"/>
+      <c r="N737" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O737" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P737" t="n">
+        <v>278</v>
+      </c>
+      <c r="Q737" t="n">
+        <v>115</v>
+      </c>
+      <c r="R737" t="n">
+        <v>393</v>
+      </c>
+      <c r="S737" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T737" t="inlineStr">
+        <is>
+          <t>1881753815</t>
+        </is>
+      </c>
+      <c r="U737" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1881753815</t>
+        </is>
+      </c>
+      <c r="V737" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>리네일</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr"/>
+      <c r="D738" t="inlineStr"/>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>0507-1348-9626</t>
+        </is>
+      </c>
+      <c r="F738" t="inlineStr"/>
+      <c r="G738" t="inlineStr">
+        <is>
+          <t>경기도 용인시 수지구 정평로 40-1 거묵상가1 2층 201호</t>
+        </is>
+      </c>
+      <c r="H738" t="inlineStr">
+        <is>
+          <t>https://pf.kakao.com/_xjZtqG</t>
+        </is>
+      </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J738" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K738" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L738" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M738" t="inlineStr"/>
+      <c r="N738" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O738" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P738" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q738" t="n">
+        <v>0</v>
+      </c>
+      <c r="R738" t="n">
+        <v>24</v>
+      </c>
+      <c r="S738" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T738" t="inlineStr">
+        <is>
+          <t>1613647201</t>
+        </is>
+      </c>
+      <c r="U738" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1613647201</t>
+        </is>
+      </c>
+      <c r="V738" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>미용실</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>꾸밈헤어&amp;네일</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>aengtori@naver.com</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr"/>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>031-335-1259</t>
+        </is>
+      </c>
+      <c r="F739" t="inlineStr"/>
+      <c r="G739" t="inlineStr">
+        <is>
+          <t>경기도 용인시 처인구 포곡읍 둔전로65번길 11 1층 안쪽 상가 꾸밈헤어&amp;네일</t>
+        </is>
+      </c>
+      <c r="H739" t="inlineStr">
+        <is>
+          <t>https://pf.kakao.com/_LdMsxb</t>
+        </is>
+      </c>
+      <c r="I739" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J739" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K739" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L739" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M739" t="inlineStr"/>
+      <c r="N739" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O739" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P739" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q739" t="n">
+        <v>0</v>
+      </c>
+      <c r="R739" t="n">
+        <v>17</v>
+      </c>
+      <c r="S739" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T739" t="inlineStr">
+        <is>
+          <t>1003645633</t>
+        </is>
+      </c>
+      <c r="U739" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1003645633</t>
+        </is>
+      </c>
+      <c r="V739" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>혠즈네일</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>naeun1210@naver.com</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr"/>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>0507-1496-7951</t>
+        </is>
+      </c>
+      <c r="F740" t="inlineStr"/>
+      <c r="G740" t="inlineStr">
+        <is>
+          <t>경기도 용인시 기흥구 흥덕2로65번길 12-9 1층 혠즈네일</t>
+        </is>
+      </c>
+      <c r="H740" t="inlineStr">
+        <is>
+          <t>http://instagram.com/hyenznail</t>
+        </is>
+      </c>
+      <c r="I740" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J740" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K740" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L740" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M740" t="inlineStr"/>
+      <c r="N740" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O740" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P740" t="n">
+        <v>280</v>
+      </c>
+      <c r="Q740" t="n">
+        <v>6</v>
+      </c>
+      <c r="R740" t="n">
+        <v>286</v>
+      </c>
+      <c r="S740" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T740" t="inlineStr">
+        <is>
+          <t>1967281250</t>
+        </is>
+      </c>
+      <c r="U740" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1967281250</t>
+        </is>
+      </c>
+      <c r="V740" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>네일드벨</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr"/>
+      <c r="D741" t="inlineStr"/>
+      <c r="E741" t="inlineStr">
+        <is>
+          <t>0507-1378-1596</t>
+        </is>
+      </c>
+      <c r="F741" t="inlineStr"/>
+      <c r="G741" t="inlineStr">
+        <is>
+          <t>경기도 수원시 영통구 반달로7번길 40 2층 223-1호</t>
+        </is>
+      </c>
+      <c r="H741" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nail.de_belle?igsh=cHNjdHAzcG9qaDho&amp;utm_source=qr</t>
+        </is>
+      </c>
+      <c r="I741" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J741" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K741" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L741" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M741" t="inlineStr"/>
+      <c r="N741" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O741" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P741" t="n">
+        <v>261</v>
+      </c>
+      <c r="Q741" t="n">
+        <v>6</v>
+      </c>
+      <c r="R741" t="n">
+        <v>267</v>
+      </c>
+      <c r="S741" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T741" t="inlineStr">
+        <is>
+          <t>1129106136</t>
+        </is>
+      </c>
+      <c r="U741" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1129106136</t>
+        </is>
+      </c>
+      <c r="V741" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>제이뷰티</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>j_beauty_lab@naver.com</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr"/>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>0507-1319-1271</t>
+        </is>
+      </c>
+      <c r="F742" t="inlineStr"/>
+      <c r="G742" t="inlineStr">
+        <is>
+          <t>경기도 용인시 처인구 한터로 159 1층 103호</t>
+        </is>
+      </c>
+      <c r="H742" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/imjeongyun187?igsh=MWh6bmZ6enV1Ynk1aA==</t>
+        </is>
+      </c>
+      <c r="I742" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J742" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K742" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L742" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M742" t="inlineStr"/>
+      <c r="N742" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O742" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P742" t="n">
+        <v>200</v>
+      </c>
+      <c r="Q742" t="n">
+        <v>17</v>
+      </c>
+      <c r="R742" t="n">
+        <v>217</v>
+      </c>
+      <c r="S742" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T742" t="inlineStr">
+        <is>
+          <t>1883484078</t>
+        </is>
+      </c>
+      <c r="U742" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1883484078</t>
+        </is>
+      </c>
+      <c r="V742" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>네일마주봄</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>prim-rose@naver.com</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr"/>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>0507-1361-5110</t>
+        </is>
+      </c>
+      <c r="F743" t="inlineStr"/>
+      <c r="G743" t="inlineStr">
+        <is>
+          <t>경기도 용인시 처인구 백옥대로 1130-1 1층 네일마주봄</t>
+        </is>
+      </c>
+      <c r="H743" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_Bxexnbxb</t>
+        </is>
+      </c>
+      <c r="I743" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J743" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K743" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L743" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M743" t="inlineStr"/>
+      <c r="N743" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O743" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P743" t="n">
+        <v>77</v>
+      </c>
+      <c r="Q743" t="n">
+        <v>54</v>
+      </c>
+      <c r="R743" t="n">
+        <v>131</v>
+      </c>
+      <c r="S743" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T743" t="inlineStr">
+        <is>
+          <t>1778117192</t>
+        </is>
+      </c>
+      <c r="U743" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1778117192</t>
+        </is>
+      </c>
+      <c r="V743" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Wnail</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>silverg0210@naver.com</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr"/>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>0507-1378-5660</t>
+        </is>
+      </c>
+      <c r="F744" t="inlineStr"/>
+      <c r="G744" t="inlineStr">
+        <is>
+          <t>경기도 용인시 수지구 광교중앙로295번길 25 a동 103호 w nail</t>
+        </is>
+      </c>
+      <c r="H744" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/w_nail4940</t>
+        </is>
+      </c>
+      <c r="I744" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J744" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K744" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L744" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M744" t="inlineStr"/>
+      <c r="N744" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O744" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P744" t="n">
+        <v>191</v>
+      </c>
+      <c r="Q744" t="n">
+        <v>2</v>
+      </c>
+      <c r="R744" t="n">
+        <v>193</v>
+      </c>
+      <c r="S744" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T744" t="inlineStr">
+        <is>
+          <t>1317247038</t>
+        </is>
+      </c>
+      <c r="U744" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1317247038</t>
+        </is>
+      </c>
+      <c r="V744" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>쁘네일래쉬</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>cptai3@naver.com</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr"/>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>0507-1370-1593</t>
+        </is>
+      </c>
+      <c r="F745" t="inlineStr"/>
+      <c r="G745" t="inlineStr">
+        <is>
+          <t>경기도 수원시 영통구 영통로331번길 70 1층</t>
+        </is>
+      </c>
+      <c r="H745" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_wGLgxj</t>
+        </is>
+      </c>
+      <c r="I745" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J745" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K745" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L745" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M745" t="inlineStr"/>
+      <c r="N745" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O745" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P745" t="n">
+        <v>108</v>
+      </c>
+      <c r="Q745" t="n">
+        <v>48</v>
+      </c>
+      <c r="R745" t="n">
+        <v>156</v>
+      </c>
+      <c r="S745" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T745" t="inlineStr">
+        <is>
+          <t>1734795951</t>
+        </is>
+      </c>
+      <c r="U745" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1734795951</t>
+        </is>
+      </c>
+      <c r="V745" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>희연네일 광교중앙역점</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>heeyeoun_nail@naver.com</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr"/>
+      <c r="E746" t="inlineStr"/>
+      <c r="F746" t="inlineStr"/>
+      <c r="G746" t="inlineStr">
+        <is>
+          <t>경기도 수원시 영통구 도청로18번길 26 1동 지하2층 B258호</t>
+        </is>
+      </c>
+      <c r="H746" t="inlineStr">
+        <is>
+          <t>https://http//pf.kakao.com/_YGkxgG</t>
+        </is>
+      </c>
+      <c r="I746" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J746" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K746" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L746" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M746" t="inlineStr"/>
+      <c r="N746" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O746" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P746" t="n">
+        <v>406</v>
+      </c>
+      <c r="Q746" t="n">
+        <v>71</v>
+      </c>
+      <c r="R746" t="n">
+        <v>477</v>
+      </c>
+      <c r="S746" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T746" t="inlineStr">
+        <is>
+          <t>1710940821</t>
+        </is>
+      </c>
+      <c r="U746" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1710940821</t>
+        </is>
+      </c>
+      <c r="V746" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>41.네일</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>jhu5239@naver.com</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr"/>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>031-266-4141</t>
+        </is>
+      </c>
+      <c r="F747" t="inlineStr"/>
+      <c r="G747" t="inlineStr">
+        <is>
+          <t>경기도 용인시 수지구 성복2로 17 골드프라자 1층 41.nail</t>
+        </is>
+      </c>
+      <c r="H747" t="inlineStr">
+        <is>
+          <t>http://instagram.com/41.nail</t>
+        </is>
+      </c>
+      <c r="I747" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J747" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K747" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L747" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M747" t="inlineStr"/>
+      <c r="N747" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O747" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P747" t="n">
+        <v>420</v>
+      </c>
+      <c r="Q747" t="n">
+        <v>16</v>
+      </c>
+      <c r="R747" t="n">
+        <v>436</v>
+      </c>
+      <c r="S747" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T747" t="inlineStr">
+        <is>
+          <t>1052711620</t>
+        </is>
+      </c>
+      <c r="U747" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1052711620</t>
+        </is>
+      </c>
+      <c r="V747" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>네일손발공주 보정점</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>miri3891@naver.com</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr"/>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>0507-1437-1469</t>
+        </is>
+      </c>
+      <c r="F748" t="inlineStr"/>
+      <c r="G748" t="inlineStr">
+        <is>
+          <t>경기도 용인시 기흥구 죽현로 8-20 아이원프라자 1층 네일손발공주</t>
+        </is>
+      </c>
+      <c r="H748" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nail_s.b.princess</t>
+        </is>
+      </c>
+      <c r="I748" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J748" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K748" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L748" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M748" t="inlineStr"/>
+      <c r="N748" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O748" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P748" t="n">
+        <v>511</v>
+      </c>
+      <c r="Q748" t="n">
+        <v>15</v>
+      </c>
+      <c r="R748" t="n">
+        <v>526</v>
+      </c>
+      <c r="S748" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T748" t="inlineStr">
+        <is>
+          <t>1798087647</t>
+        </is>
+      </c>
+      <c r="U748" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1798087647</t>
+        </is>
+      </c>
+      <c r="V748" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>네일앤코</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr"/>
+      <c r="D749" t="inlineStr"/>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>070-5100-0616</t>
+        </is>
+      </c>
+      <c r="F749" t="inlineStr"/>
+      <c r="G749" t="inlineStr">
+        <is>
+          <t>경기도 수원시 영통구 센트럴파크로127번길 131-3 1층 101호</t>
+        </is>
+      </c>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nail._.ko?igsh=OGwweW53NnNtNnl6&amp;utm_source=qr</t>
+        </is>
+      </c>
+      <c r="I749" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J749" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K749" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L749" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M749" t="inlineStr"/>
+      <c r="N749" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O749" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P749" t="n">
+        <v>327</v>
+      </c>
+      <c r="Q749" t="n">
+        <v>6</v>
+      </c>
+      <c r="R749" t="n">
+        <v>333</v>
+      </c>
+      <c r="S749" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T749" t="inlineStr">
+        <is>
+          <t>1872894083</t>
+        </is>
+      </c>
+      <c r="U749" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1872894083</t>
+        </is>
+      </c>
+      <c r="V749" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>온앤온네일</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>kimjieun514@naver.com</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr"/>
+      <c r="E750" t="inlineStr"/>
+      <c r="F750" t="inlineStr"/>
+      <c r="G750" t="inlineStr">
+        <is>
+          <t>경기도 화성시 동탄구 동탄순환대로 263 1층 111호</t>
+        </is>
+      </c>
+      <c r="H750" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/on.on_nail</t>
+        </is>
+      </c>
+      <c r="I750" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J750" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K750" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L750" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M750" t="inlineStr"/>
+      <c r="N750" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O750" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P750" t="n">
+        <v>272</v>
+      </c>
+      <c r="Q750" t="n">
+        <v>88</v>
+      </c>
+      <c r="R750" t="n">
+        <v>360</v>
+      </c>
+      <c r="S750" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T750" t="inlineStr">
+        <is>
+          <t>1997573833</t>
+        </is>
+      </c>
+      <c r="U750" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1997573833</t>
+        </is>
+      </c>
+      <c r="V750" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>미용실</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>함스헤어</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>rose74741@naver.com</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr"/>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>0507-1374-7910</t>
+        </is>
+      </c>
+      <c r="F751" t="inlineStr"/>
+      <c r="G751" t="inlineStr">
+        <is>
+          <t>경기도 용인시 처인구 유림로 148-4</t>
+        </is>
+      </c>
+      <c r="H751" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I751" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J751" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K751" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L751" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M751" t="inlineStr"/>
+      <c r="N751" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O751" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P751" t="n">
+        <v>37</v>
+      </c>
+      <c r="Q751" t="n">
+        <v>0</v>
+      </c>
+      <c r="R751" t="n">
+        <v>37</v>
+      </c>
+      <c r="S751" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T751" t="inlineStr">
+        <is>
+          <t>37036591</t>
+        </is>
+      </c>
+      <c r="U751" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/37036591</t>
+        </is>
+      </c>
+      <c r="V751" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>인테리어디자인</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>스페이스와이 SPACE Y</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>yonseiblog@naver.com</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr"/>
+      <c r="E752" t="inlineStr">
+        <is>
+          <t>0507-1396-3851</t>
+        </is>
+      </c>
+      <c r="F752" t="inlineStr"/>
+      <c r="G752" t="inlineStr">
+        <is>
+          <t>경기도 화성시 동탄구 동탄대로 599 303호</t>
+        </is>
+      </c>
+      <c r="H752" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I752" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J752" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K752" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L752" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M752" t="inlineStr"/>
+      <c r="N752" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O752" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P752" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q752" t="n">
+        <v>0</v>
+      </c>
+      <c r="R752" t="n">
+        <v>0</v>
+      </c>
+      <c r="S752" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T752" t="inlineStr">
+        <is>
+          <t>1315149633</t>
+        </is>
+      </c>
+      <c r="U752" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1315149633</t>
+        </is>
+      </c>
+      <c r="V752" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>인테리어디자인</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>웰디자인</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr"/>
+      <c r="D753" t="inlineStr"/>
+      <c r="E753" t="inlineStr"/>
+      <c r="F753" t="inlineStr"/>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>경기도 용인시 수지구 풍덕천로 52</t>
+        </is>
+      </c>
+      <c r="H753" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/well_design24</t>
+        </is>
+      </c>
+      <c r="I753" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J753" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K753" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L753" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M753" t="inlineStr"/>
+      <c r="N753" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O753" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P753" t="n">
         <v>1</v>
       </c>
-      <c r="S727" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="T727" t="inlineStr">
+      <c r="Q753" t="n">
+        <v>0</v>
+      </c>
+      <c r="R753" t="n">
+        <v>1</v>
+      </c>
+      <c r="S753" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T753" t="inlineStr">
         <is>
           <t>1956094235</t>
         </is>
       </c>
-      <c r="U727" t="inlineStr">
+      <c r="U753" t="inlineStr">
         <is>
           <t>https://m.place.naver.com/place/1956094235</t>
         </is>
       </c>
-      <c r="V727" t="inlineStr">
+      <c r="V753" t="inlineStr">
         <is>
           <t>2026-04-29</t>
         </is>

</xml_diff>